<commit_message>
add URTA + CRTA
</commit_message>
<xml_diff>
--- a/data/datasets/features/cleaned_feature_group_1.xlsx
+++ b/data/datasets/features/cleaned_feature_group_1.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,12 +450,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>std_rate[t]</t>
+          <t>mean_rate[t]</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>mean_rate[t-1]</t>
+          <t>std_rate[t]</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -485,15 +485,10 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>mean_close[t]</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>return_moex[t]</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>std_return_moex[t]</t>
         </is>
@@ -509,9 +504,11 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>7.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>8.460000000000001</v>
@@ -526,12 +523,9 @@
         <v>0.008014374198942242</v>
       </c>
       <c r="L2" t="n">
-        <v>2378.272380952381</v>
+        <v>0.01405907609363677</v>
       </c>
       <c r="M2" t="n">
-        <v>0.01405907609363677</v>
-      </c>
-      <c r="N2" t="n">
         <v>0.01004602788358254</v>
       </c>
     </row>
@@ -547,10 +541,10 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
+        <v>7.625</v>
+      </c>
+      <c r="F3" t="n">
         <v>0.1282472940106444</v>
-      </c>
-      <c r="F3" t="n">
-        <v>7.5</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -568,12 +562,9 @@
         <v>0.008130777007981038</v>
       </c>
       <c r="L3" t="n">
-        <v>2372.620476190476</v>
+        <v>-0.02943646336417904</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.02943646336417904</v>
-      </c>
-      <c r="N3" t="n">
         <v>0.00912830584663935</v>
       </c>
     </row>
@@ -591,10 +582,10 @@
         <v>-0.003659841606166059</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="F4" t="n">
-        <v>7.625</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>0.1282472940106444</v>
@@ -612,12 +603,9 @@
         <v>0.008028646452857391</v>
       </c>
       <c r="L4" t="n">
-        <v>2455.88</v>
+        <v>0.0612476847954202</v>
       </c>
       <c r="M4" t="n">
-        <v>0.0612476847954202</v>
-      </c>
-      <c r="N4" t="n">
         <v>0.006080206265164916</v>
       </c>
     </row>
@@ -635,10 +623,10 @@
         <v>-0.005258373066935773</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="F5" t="n">
-        <v>7.75</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -656,12 +644,9 @@
         <v>0.008406167604495085</v>
       </c>
       <c r="L5" t="n">
-        <v>2498.371</v>
+        <v>-0.01444660348177806</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.01444660348177806</v>
-      </c>
-      <c r="N5" t="n">
         <v>0.008159771950762602</v>
       </c>
     </row>
@@ -679,10 +664,10 @@
         <v>0.000803082835922897</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="F6" t="n">
-        <v>7.75</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -700,12 +685,9 @@
         <v>0.007983990555842979</v>
       </c>
       <c r="L6" t="n">
-        <v>2484.8475</v>
+        <v>0.00770376229313019</v>
       </c>
       <c r="M6" t="n">
-        <v>0.00770376229313019</v>
-      </c>
-      <c r="N6" t="n">
         <v>0.005283095376779708</v>
       </c>
     </row>
@@ -723,10 +705,10 @@
         <v>0.00200021571012865</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="F7" t="n">
-        <v>7.75</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -744,12 +726,9 @@
         <v>0.008391878006036579</v>
       </c>
       <c r="L7" t="n">
-        <v>2558.224090909091</v>
+        <v>0.01509965294992566</v>
       </c>
       <c r="M7" t="n">
-        <v>0.01509965294992566</v>
-      </c>
-      <c r="N7" t="n">
         <v>0.004989975440526886</v>
       </c>
     </row>
@@ -767,10 +746,10 @@
         <v>0.002111402467871892</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>7.75</v>
       </c>
       <c r="F8" t="n">
-        <v>7.75</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -788,12 +767,9 @@
         <v>0.008295288815264312</v>
       </c>
       <c r="L8" t="n">
-        <v>2591.336666666667</v>
+        <v>0.03499118521912692</v>
       </c>
       <c r="M8" t="n">
-        <v>0.03499118521912692</v>
-      </c>
-      <c r="N8" t="n">
         <v>0.008706731602258148</v>
       </c>
     </row>
@@ -811,10 +787,10 @@
         <v>0.001501934960091322</v>
       </c>
       <c r="E9" t="n">
+        <v>7.625</v>
+      </c>
+      <c r="F9" t="n">
         <v>0.1282472940106444</v>
-      </c>
-      <c r="F9" t="n">
-        <v>7.75</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -832,12 +808,9 @@
         <v>0.008156615765260833</v>
       </c>
       <c r="L9" t="n">
-        <v>2748.511052631579</v>
+        <v>0.01315784653818963</v>
       </c>
       <c r="M9" t="n">
-        <v>0.01315784653818963</v>
-      </c>
-      <c r="N9" t="n">
         <v>0.007745725598663074</v>
       </c>
     </row>
@@ -855,10 +828,10 @@
         <v>0.004481556380874219</v>
       </c>
       <c r="E10" t="n">
+        <v>7.467391304347826</v>
+      </c>
+      <c r="F10" t="n">
         <v>0.08608755539377277</v>
-      </c>
-      <c r="F10" t="n">
-        <v>7.625</v>
       </c>
       <c r="G10" t="n">
         <v>0.1282472940106444</v>
@@ -876,12 +849,9 @@
         <v>0.007901033147613035</v>
       </c>
       <c r="L10" t="n">
-        <v>2759.329565217392</v>
+        <v>-0.0221205295791137</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.0221205295791137</v>
-      </c>
-      <c r="N10" t="n">
         <v>0.006620373888041498</v>
       </c>
     </row>
@@ -899,10 +869,10 @@
         <v>0.00263289982888093</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>7.25</v>
       </c>
       <c r="F11" t="n">
-        <v>7.467391304347826</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0.08608755539377277</v>
@@ -920,12 +890,9 @@
         <v>0.007994450384145146</v>
       </c>
       <c r="L11" t="n">
-        <v>2673.455454545454</v>
+        <v>0.003890936535967393</v>
       </c>
       <c r="M11" t="n">
-        <v>0.003890936535967393</v>
-      </c>
-      <c r="N11" t="n">
         <v>0.009023169856437382</v>
       </c>
     </row>
@@ -943,10 +910,10 @@
         <v>0.006999509255407821</v>
       </c>
       <c r="E12" t="n">
+        <v>7.059523809523809</v>
+      </c>
+      <c r="F12" t="n">
         <v>0.1091089451179959</v>
-      </c>
-      <c r="F12" t="n">
-        <v>7.25</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -964,12 +931,9 @@
         <v>0.007872293733319324</v>
       </c>
       <c r="L12" t="n">
-        <v>2789.105238095238</v>
+        <v>-0.009314787901955057</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.009314787901955057</v>
-      </c>
-      <c r="N12" t="n">
         <v>0.006837605387753504</v>
       </c>
     </row>
@@ -987,10 +951,10 @@
         <v>0.006073481927781677</v>
       </c>
       <c r="E13" t="n">
+        <v>6.913043478260869</v>
+      </c>
+      <c r="F13" t="n">
         <v>0.1937766939407946</v>
-      </c>
-      <c r="F13" t="n">
-        <v>7.059523809523809</v>
       </c>
       <c r="G13" t="n">
         <v>0.1091089451179959</v>
@@ -1008,12 +972,9 @@
         <v>0.007485499461442169</v>
       </c>
       <c r="L13" t="n">
-        <v>2773.500434782609</v>
+        <v>0.04898815802351009</v>
       </c>
       <c r="M13" t="n">
-        <v>0.04898815802351009</v>
-      </c>
-      <c r="N13" t="n">
         <v>0.007967135324941178</v>
       </c>
     </row>
@@ -1031,10 +992,10 @@
         <v>0.003104167702907557</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="F14" t="n">
-        <v>6.913043478260869</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
         <v>0.1937766939407946</v>
@@ -1052,12 +1013,9 @@
         <v>0.006960347917780219</v>
       </c>
       <c r="L14" t="n">
-        <v>2945.8575</v>
+        <v>0.001696014196014062</v>
       </c>
       <c r="M14" t="n">
-        <v>0.001696014196014062</v>
-      </c>
-      <c r="N14" t="n">
         <v>0.006341854216422482</v>
       </c>
     </row>
@@ -1075,10 +1033,10 @@
         <v>0.001246723300462049</v>
       </c>
       <c r="E15" t="n">
+        <v>6.363636363636363</v>
+      </c>
+      <c r="F15" t="n">
         <v>0.1274117978594065</v>
-      </c>
-      <c r="F15" t="n">
-        <v>6.5</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -1096,12 +1054,9 @@
         <v>0.007501542999799549</v>
       </c>
       <c r="L15" t="n">
-        <v>2982.649047619047</v>
+        <v>0.04268480545532971</v>
       </c>
       <c r="M15" t="n">
-        <v>0.04268480545532971</v>
-      </c>
-      <c r="N15" t="n">
         <v>0.005569115925732852</v>
       </c>
     </row>
@@ -1119,10 +1074,10 @@
         <v>0.0005359229477224225</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="F16" t="n">
-        <v>6.363636363636363</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
         <v>0.1274117978594065</v>
@@ -1140,12 +1095,9 @@
         <v>0.006872361604873811</v>
       </c>
       <c r="L16" t="n">
-        <v>3133.9345</v>
+        <v>9.101636019082093e-05</v>
       </c>
       <c r="M16" t="n">
-        <v>9.101636019082093e-05</v>
-      </c>
-      <c r="N16" t="n">
         <v>0.008826972650268316</v>
       </c>
     </row>
@@ -1163,10 +1115,10 @@
         <v>-5.325381257659245e-05</v>
       </c>
       <c r="E17" t="n">
+        <v>6.065789473684211</v>
+      </c>
+      <c r="F17" t="n">
         <v>0.1131034820897157</v>
-      </c>
-      <c r="F17" t="n">
-        <v>6.25</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1184,12 +1136,9 @@
         <v>0.007011987926942798</v>
       </c>
       <c r="L17" t="n">
-        <v>3063.527368421053</v>
+        <v>-0.09305597165596391</v>
       </c>
       <c r="M17" t="n">
-        <v>-0.09305597165596391</v>
-      </c>
-      <c r="N17" t="n">
         <v>0.01598529435161526</v>
       </c>
     </row>
@@ -1207,10 +1156,10 @@
         <v>0.0004373739016456657</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
-        <v>6.065789473684211</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>0.1131034820897157</v>
@@ -1228,12 +1177,9 @@
         <v>0.006675070138181471</v>
       </c>
       <c r="L18" t="n">
-        <v>2462.514285714286</v>
+        <v>-0.09290721932770984</v>
       </c>
       <c r="M18" t="n">
-        <v>-0.09290721932770984</v>
-      </c>
-      <c r="N18" t="n">
         <v>0.04125177412267202</v>
       </c>
     </row>
@@ -1251,10 +1197,10 @@
         <v>-0.001719737122258924</v>
       </c>
       <c r="E19" t="n">
+        <v>5.909090909090909</v>
+      </c>
+      <c r="F19" t="n">
         <v>0.1973855084879308</v>
-      </c>
-      <c r="F19" t="n">
-        <v>6</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1272,12 +1218,9 @@
         <v>0.006675070138181471</v>
       </c>
       <c r="L19" t="n">
-        <v>2588.827272727272</v>
+        <v>0.07153512477714741</v>
       </c>
       <c r="M19" t="n">
-        <v>0.07153512477714741</v>
-      </c>
-      <c r="N19" t="n">
         <v>0.0185084518405279</v>
       </c>
     </row>
@@ -1295,10 +1238,10 @@
         <v>-0.004048943404469929</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="F20" t="n">
-        <v>5.909090909090909</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0.1973855084879308</v>
@@ -1316,12 +1259,9 @@
         <v>0.006675070138181471</v>
       </c>
       <c r="L20" t="n">
-        <v>2683.665789473684</v>
+        <v>0.04198290051207021</v>
       </c>
       <c r="M20" t="n">
-        <v>0.04198290051207021</v>
-      </c>
-      <c r="N20" t="n">
         <v>0.01424545364565375</v>
       </c>
     </row>
@@ -1339,10 +1279,10 @@
         <v>0.0008763472392376848</v>
       </c>
       <c r="E21" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F21" t="n">
         <v>0.4701623459816271</v>
-      </c>
-      <c r="F21" t="n">
-        <v>5.5</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1360,12 +1300,9 @@
         <v>0.006675070138181471</v>
       </c>
       <c r="L21" t="n">
-        <v>2766.8685</v>
+        <v>-0.002559776601314789</v>
       </c>
       <c r="M21" t="n">
-        <v>-0.002559776601314789</v>
-      </c>
-      <c r="N21" t="n">
         <v>0.01035748406756849</v>
       </c>
     </row>
@@ -1383,10 +1320,10 @@
         <v>0.001263693147037115</v>
       </c>
       <c r="E22" t="n">
+        <v>4.443181818181818</v>
+      </c>
+      <c r="F22" t="n">
         <v>0.1072330068072219</v>
-      </c>
-      <c r="F22" t="n">
-        <v>5.2</v>
       </c>
       <c r="G22" t="n">
         <v>0.4701623459816271</v>
@@ -1404,12 +1341,9 @@
         <v>0.006675070138181471</v>
       </c>
       <c r="L22" t="n">
-        <v>2823.388181818182</v>
+        <v>0.04402626228579432</v>
       </c>
       <c r="M22" t="n">
-        <v>0.04402626228579432</v>
-      </c>
-      <c r="N22" t="n">
         <v>0.008053728349225221</v>
       </c>
     </row>
@@ -1427,10 +1361,10 @@
         <v>-0.0004018844810861344</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F23" t="n">
-        <v>4.443181818181818</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>0.1072330068072219</v>
@@ -1448,12 +1382,9 @@
         <v>0.007353590312176195</v>
       </c>
       <c r="L23" t="n">
-        <v>3009.748095238095</v>
+        <v>0.01236531432062438</v>
       </c>
       <c r="M23" t="n">
-        <v>0.01236531432062438</v>
-      </c>
-      <c r="N23" t="n">
         <v>0.009806834682388852</v>
       </c>
     </row>
@@ -1471,10 +1402,10 @@
         <v>0.003320661985517503</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F24" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1492,12 +1423,9 @@
         <v>0.007529631614800802</v>
       </c>
       <c r="L24" t="n">
-        <v>2923.413181818182</v>
+        <v>-0.02325714285714287</v>
       </c>
       <c r="M24" t="n">
-        <v>-0.02325714285714287</v>
-      </c>
-      <c r="N24" t="n">
         <v>0.009973711920105004</v>
       </c>
     </row>
@@ -1515,10 +1443,10 @@
         <v>0.003646093841701115</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F25" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1536,12 +1464,9 @@
         <v>0.007678909222941233</v>
       </c>
       <c r="L25" t="n">
-        <v>2810.621363636364</v>
+        <v>-0.06893556647518861</v>
       </c>
       <c r="M25" t="n">
-        <v>-0.06893556647518861</v>
-      </c>
-      <c r="N25" t="n">
         <v>0.009155876774330919</v>
       </c>
     </row>
@@ -1559,10 +1484,10 @@
         <v>-0.001294432351477415</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F26" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1580,12 +1505,9 @@
         <v>0.008533080028072959</v>
       </c>
       <c r="L26" t="n">
-        <v>3015.494</v>
+        <v>0.1351724541011272</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1351724541011272</v>
-      </c>
-      <c r="N26" t="n">
         <v>0.01181724354630124</v>
       </c>
     </row>
@@ -1603,10 +1525,10 @@
         <v>-0.004247405449129826</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F27" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1624,12 +1546,9 @@
         <v>0.009454611167698079</v>
       </c>
       <c r="L27" t="n">
-        <v>3232.552272727272</v>
+        <v>0.04486639833025707</v>
       </c>
       <c r="M27" t="n">
-        <v>0.04486639833025707</v>
-      </c>
-      <c r="N27" t="n">
         <v>0.009454015132036631</v>
       </c>
     </row>
@@ -1647,10 +1566,10 @@
         <v>-0.005304364342932133</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F28" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1668,12 +1587,9 @@
         <v>0.01010361404333815</v>
       </c>
       <c r="L28" t="n">
-        <v>3412.641578947369</v>
+        <v>-0.0219160665092778</v>
       </c>
       <c r="M28" t="n">
-        <v>-0.0219160665092778</v>
-      </c>
-      <c r="N28" t="n">
         <v>0.01122580479597159</v>
       </c>
     </row>
@@ -1691,10 +1607,10 @@
         <v>-0.003763521399523406</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>4.25</v>
       </c>
       <c r="F29" t="n">
-        <v>4.25</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
         <v>0</v>
@@ -1712,12 +1628,9 @@
         <v>0.009702759251767334</v>
       </c>
       <c r="L29" t="n">
-        <v>3408.367</v>
+        <v>0.01686345764689445</v>
       </c>
       <c r="M29" t="n">
-        <v>0.01686345764689445</v>
-      </c>
-      <c r="N29" t="n">
         <v>0.01149096205029011</v>
       </c>
     </row>
@@ -1735,10 +1648,10 @@
         <v>-0.004987148788045959</v>
       </c>
       <c r="E30" t="n">
+        <v>4.340909090909091</v>
+      </c>
+      <c r="F30" t="n">
         <v>0.1230914909793327</v>
-      </c>
-      <c r="F30" t="n">
-        <v>4.25</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1756,12 +1669,9 @@
         <v>0.009981994816071982</v>
       </c>
       <c r="L30" t="n">
-        <v>3483.779090909091</v>
+        <v>0.04593994377111543</v>
       </c>
       <c r="M30" t="n">
-        <v>0.04593994377111543</v>
-      </c>
-      <c r="N30" t="n">
         <v>0.01000652322859552</v>
       </c>
     </row>
@@ -1779,10 +1689,10 @@
         <v>-0.003728718889754234</v>
       </c>
       <c r="E31" t="n">
+        <v>4.613636363636363</v>
+      </c>
+      <c r="F31" t="n">
         <v>0.2144660136144444</v>
-      </c>
-      <c r="F31" t="n">
-        <v>4.340909090909091</v>
       </c>
       <c r="G31" t="n">
         <v>0.1230914909793327</v>
@@ -1800,12 +1710,9 @@
         <v>0.01138353379333767</v>
       </c>
       <c r="L31" t="n">
-        <v>3553.729545454546</v>
+        <v>0.004666141276923774</v>
       </c>
       <c r="M31" t="n">
-        <v>0.004666141276923774</v>
-      </c>
-      <c r="N31" t="n">
         <v>0.006994927293485055</v>
       </c>
     </row>
@@ -1823,10 +1730,10 @@
         <v>-0.002759805090574718</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
-        <v>4.613636363636363</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
         <v>0.2144660136144444</v>
@@ -1844,12 +1751,9 @@
         <v>0.01157316765141214</v>
       </c>
       <c r="L32" t="n">
-        <v>3667.3915</v>
+        <v>0.04037224540913176</v>
       </c>
       <c r="M32" t="n">
-        <v>0.04037224540913176</v>
-      </c>
-      <c r="N32" t="n">
         <v>0.007674785173122899</v>
       </c>
     </row>
@@ -1867,10 +1771,10 @@
         <v>-0.004535917656929178</v>
       </c>
       <c r="E33" t="n">
+        <v>5.272727272727272</v>
+      </c>
+      <c r="F33" t="n">
         <v>0.2548235957188125</v>
-      </c>
-      <c r="F33" t="n">
-        <v>5</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1888,12 +1792,9 @@
         <v>0.01166534419414322</v>
       </c>
       <c r="L33" t="n">
-        <v>3820.791363636364</v>
+        <v>0.0205228192180289</v>
       </c>
       <c r="M33" t="n">
-        <v>0.0205228192180289</v>
-      </c>
-      <c r="N33" t="n">
         <v>0.006561863746099084</v>
       </c>
     </row>
@@ -1911,10 +1812,10 @@
         <v>-0.003929345937022544</v>
       </c>
       <c r="E34" t="n">
+        <v>5.727272727272728</v>
+      </c>
+      <c r="F34" t="n">
         <v>0.4289320272288887</v>
-      </c>
-      <c r="F34" t="n">
-        <v>5.272727272727272</v>
       </c>
       <c r="G34" t="n">
         <v>0.2548235957188125</v>
@@ -1932,12 +1833,9 @@
         <v>0.01282243045693265</v>
       </c>
       <c r="L34" t="n">
-        <v>3804.949090909091</v>
+        <v>-0.02248128719235321</v>
       </c>
       <c r="M34" t="n">
-        <v>-0.02248128719235321</v>
-      </c>
-      <c r="N34" t="n">
         <v>0.00778794830354564</v>
       </c>
     </row>
@@ -1955,10 +1853,10 @@
         <v>8.500379651099621e-05</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="F35" t="n">
-        <v>5.727272727272728</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
         <v>0.4289320272288887</v>
@@ -1976,12 +1874,9 @@
         <v>0.01280352281223962</v>
       </c>
       <c r="L35" t="n">
-        <v>3866.512727272727</v>
+        <v>0.03454502257068182</v>
       </c>
       <c r="M35" t="n">
-        <v>0.03454502257068182</v>
-      </c>
-      <c r="N35" t="n">
         <v>0.007682772516184841</v>
       </c>
     </row>
@@ -1999,10 +1894,10 @@
         <v>0.001763475363841804</v>
       </c>
       <c r="E36" t="n">
+        <v>6.659090909090909</v>
+      </c>
+      <c r="F36" t="n">
         <v>0.1230914909793325</v>
-      </c>
-      <c r="F36" t="n">
-        <v>6.5</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -2020,12 +1915,9 @@
         <v>0.0121552038504491</v>
       </c>
       <c r="L36" t="n">
-        <v>4028.552727272727</v>
+        <v>0.03336674204612433</v>
       </c>
       <c r="M36" t="n">
-        <v>0.03336674204612433</v>
-      </c>
-      <c r="N36" t="n">
         <v>0.007402591237495392</v>
       </c>
     </row>
@@ -2043,10 +1935,10 @@
         <v>-0.002359071530727008</v>
       </c>
       <c r="E37" t="n">
+        <v>6.928571428571429</v>
+      </c>
+      <c r="F37" t="n">
         <v>0.3273268353539887</v>
-      </c>
-      <c r="F37" t="n">
-        <v>6.659090909090909</v>
       </c>
       <c r="G37" t="n">
         <v>0.1230914909793325</v>
@@ -2064,12 +1956,9 @@
         <v>0.01263796951416052</v>
       </c>
       <c r="L37" t="n">
-        <v>4221.789047619048</v>
+        <v>0.01541721413558639</v>
       </c>
       <c r="M37" t="n">
-        <v>0.01541721413558639</v>
-      </c>
-      <c r="N37" t="n">
         <v>0.01000598201961041</v>
       </c>
     </row>
@@ -2087,10 +1976,10 @@
         <v>-0.007209205397732399</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F38" t="n">
-        <v>6.928571428571429</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
         <v>0.3273268353539887</v>
@@ -2108,12 +1997,9 @@
         <v>0.01257850653964399</v>
       </c>
       <c r="L38" t="n">
-        <v>4071.658095238095</v>
+        <v>-0.07838464617942942</v>
       </c>
       <c r="M38" t="n">
-        <v>-0.07838464617942942</v>
-      </c>
-      <c r="N38" t="n">
         <v>0.01508263712784057</v>
       </c>
     </row>
@@ -2131,10 +2017,10 @@
         <v>-0.005489119742878801</v>
       </c>
       <c r="E39" t="n">
+        <v>7.909090909090909</v>
+      </c>
+      <c r="F39" t="n">
         <v>0.5032362797401966</v>
-      </c>
-      <c r="F39" t="n">
-        <v>7.5</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -2152,12 +2038,9 @@
         <v>0.01365090615250653</v>
       </c>
       <c r="L39" t="n">
-        <v>3761.187727272727</v>
+        <v>-0.04344970941759752</v>
       </c>
       <c r="M39" t="n">
-        <v>-0.04344970941759752</v>
-      </c>
-      <c r="N39" t="n">
         <v>0.01701681202968913</v>
       </c>
     </row>
@@ -2175,10 +2058,10 @@
         <v>-0.004052807675662518</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="F40" t="n">
-        <v>7.909090909090909</v>
+        <v>0</v>
       </c>
       <c r="G40" t="n">
         <v>0.5032362797401966</v>
@@ -2196,12 +2079,9 @@
         <v>0.0129564836441014</v>
       </c>
       <c r="L40" t="n">
-        <v>3585.712857142857</v>
+        <v>-0.0836132381570408</v>
       </c>
       <c r="M40" t="n">
-        <v>-0.0836132381570408</v>
-      </c>
-      <c r="N40" t="n">
         <v>0.0274639282932512</v>
       </c>
     </row>
@@ -2219,10 +2099,10 @@
         <v>-0.005784548264591183</v>
       </c>
       <c r="E41" t="n">
+        <v>9.574999999999999</v>
+      </c>
+      <c r="F41" t="n">
         <v>2.504075625224227</v>
-      </c>
-      <c r="F41" t="n">
-        <v>8.5</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -2240,12 +2120,9 @@
         <v>0.01327368363582493</v>
       </c>
       <c r="L41" t="n">
-        <v>3343.366111111111</v>
+        <v>-0.3037312191918651</v>
       </c>
       <c r="M41" t="n">
-        <v>-0.3037312191918651</v>
-      </c>
-      <c r="N41" t="n">
         <v>0.09856781205616666</v>
       </c>
     </row>
@@ -2263,10 +2140,10 @@
         <v>-0.006597398301041668</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F42" t="n">
-        <v>9.574999999999999</v>
+        <v>0</v>
       </c>
       <c r="G42" t="n">
         <v>2.504075625224227</v>
@@ -2284,12 +2161,9 @@
         <v>0.01267251155110927</v>
       </c>
       <c r="L42" t="n">
-        <v>2519.728333333333</v>
+        <v>0.04847760916188038</v>
       </c>
       <c r="M42" t="n">
-        <v>0.04847760916188038</v>
-      </c>
-      <c r="N42" t="n">
         <v>0.04450020546967962</v>
       </c>
     </row>
@@ -2307,10 +2181,10 @@
         <v>-0.05915329623667553</v>
       </c>
       <c r="E43" t="n">
+        <v>17.85714285714286</v>
+      </c>
+      <c r="F43" t="n">
         <v>1.388730149658827</v>
-      </c>
-      <c r="F43" t="n">
-        <v>20</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -2328,12 +2202,9 @@
         <v>0.01525601025807743</v>
       </c>
       <c r="L43" t="n">
-        <v>2464.659047619048</v>
+        <v>-0.1139532692670058</v>
       </c>
       <c r="M43" t="n">
-        <v>-0.1139532692670058</v>
-      </c>
-      <c r="N43" t="n">
         <v>0.02732218260522392</v>
       </c>
     </row>
@@ -2351,10 +2222,10 @@
         <v>-0.007561370955160185</v>
       </c>
       <c r="E44" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F44" t="n">
         <v>1.150447483271056</v>
-      </c>
-      <c r="F44" t="n">
-        <v>17.85714285714286</v>
       </c>
       <c r="G44" t="n">
         <v>1.388730149658827</v>
@@ -2372,12 +2243,9 @@
         <v>0.01883213580030252</v>
       </c>
       <c r="L44" t="n">
-        <v>2373.321666666667</v>
+        <v>-0.007336209947917505</v>
       </c>
       <c r="M44" t="n">
-        <v>-0.007336209947917505</v>
-      </c>
-      <c r="N44" t="n">
         <v>0.02043265301419003</v>
       </c>
     </row>
@@ -2395,10 +2263,10 @@
         <v>0.003702598420850522</v>
       </c>
       <c r="E45" t="n">
+        <v>10.07142857142857</v>
+      </c>
+      <c r="F45" t="n">
         <v>0.746420027292179</v>
-      </c>
-      <c r="F45" t="n">
-        <v>13.5</v>
       </c>
       <c r="G45" t="n">
         <v>1.150447483271056</v>
@@ -2416,12 +2284,9 @@
         <v>0.01788860903783429</v>
       </c>
       <c r="L45" t="n">
-        <v>2341.398571428571</v>
+        <v>-0.07148572391139563</v>
       </c>
       <c r="M45" t="n">
-        <v>-0.07148572391139563</v>
-      </c>
-      <c r="N45" t="n">
         <v>0.02007041179296356</v>
       </c>
     </row>
@@ -2439,10 +2304,10 @@
         <v>0.009421786158348544</v>
       </c>
       <c r="E46" t="n">
+        <v>9.142857142857142</v>
+      </c>
+      <c r="F46" t="n">
         <v>0.6546536707079774</v>
-      </c>
-      <c r="F46" t="n">
-        <v>10.07142857142857</v>
       </c>
       <c r="G46" t="n">
         <v>0.746420027292179</v>
@@ -2460,12 +2325,9 @@
         <v>0.01683222012101293</v>
       </c>
       <c r="L46" t="n">
-        <v>2150.736190476191</v>
+        <v>0.003262923670245277</v>
       </c>
       <c r="M46" t="n">
-        <v>0.003262923670245277</v>
-      </c>
-      <c r="N46" t="n">
         <v>0.01472871772618316</v>
       </c>
     </row>
@@ -2483,10 +2345,10 @@
         <v>0.008968274331833781</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
-        <v>9.142857142857142</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
         <v>0.6546536707079774</v>
@@ -2504,12 +2366,9 @@
         <v>0.01568198511428576</v>
       </c>
       <c r="L47" t="n">
-        <v>2194.585652173913</v>
+        <v>0.1009086780820974</v>
       </c>
       <c r="M47" t="n">
-        <v>0.1009086780820974</v>
-      </c>
-      <c r="N47" t="n">
         <v>0.01527250356872139</v>
       </c>
     </row>
@@ -2527,10 +2386,10 @@
         <v>0.01005662392080331</v>
       </c>
       <c r="E48" t="n">
+        <v>7.772727272727272</v>
+      </c>
+      <c r="F48" t="n">
         <v>0.2548235957188127</v>
-      </c>
-      <c r="F48" t="n">
-        <v>8</v>
       </c>
       <c r="G48" t="n">
         <v>0</v>
@@ -2548,12 +2407,9 @@
         <v>0.01637208664483558</v>
       </c>
       <c r="L48" t="n">
-        <v>2276.477272727273</v>
+        <v>-0.1997162447818069</v>
       </c>
       <c r="M48" t="n">
-        <v>-0.1997162447818069</v>
-      </c>
-      <c r="N48" t="n">
         <v>0.02923209834093561</v>
       </c>
     </row>
@@ -2571,10 +2427,10 @@
         <v>0.004460070203243571</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F49" t="n">
-        <v>7.772727272727272</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
         <v>0.2548235957188127</v>
@@ -2592,12 +2448,9 @@
         <v>0.01406326044273043</v>
       </c>
       <c r="L49" t="n">
-        <v>2034.042857142857</v>
+        <v>0.06104429077944729</v>
       </c>
       <c r="M49" t="n">
-        <v>0.06104429077944729</v>
-      </c>
-      <c r="N49" t="n">
         <v>0.01922782870904712</v>
       </c>
     </row>
@@ -2615,10 +2468,10 @@
         <v>0.002975254824195916</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F50" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -2636,12 +2489,9 @@
         <v>0.01362340760317871</v>
       </c>
       <c r="L50" t="n">
-        <v>2197.44</v>
+        <v>8.278336054456936e-05</v>
       </c>
       <c r="M50" t="n">
-        <v>8.278336054456936e-05</v>
-      </c>
-      <c r="N50" t="n">
         <v>0.01107646859560671</v>
       </c>
     </row>
@@ -2659,10 +2509,10 @@
         <v>0.001296951564024207</v>
       </c>
       <c r="E51" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F51" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -2680,12 +2530,9 @@
         <v>0.0126583624938903</v>
       </c>
       <c r="L51" t="n">
-        <v>2156.263636363637</v>
+        <v>-0.01516488440033104</v>
       </c>
       <c r="M51" t="n">
-        <v>-0.01516488440033104</v>
-      </c>
-      <c r="N51" t="n">
         <v>0.005857695718131788</v>
       </c>
     </row>
@@ -2703,10 +2550,10 @@
         <v>-0.002964641292140024</v>
       </c>
       <c r="E52" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F52" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -2724,12 +2571,9 @@
         <v>0.01160510231102285</v>
       </c>
       <c r="L52" t="n">
-        <v>2181.810952380952</v>
+        <v>0.02435701529907774</v>
       </c>
       <c r="M52" t="n">
-        <v>0.02435701529907774</v>
-      </c>
-      <c r="N52" t="n">
         <v>0.007329908801977214</v>
       </c>
     </row>
@@ -2747,10 +2591,10 @@
         <v>-0.003785491438719868</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F53" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -2768,12 +2612,9 @@
         <v>0.01172474029370796</v>
       </c>
       <c r="L53" t="n">
-        <v>2228.133157894737</v>
+        <v>0.01031769163509177</v>
       </c>
       <c r="M53" t="n">
-        <v>0.01031769163509177</v>
-      </c>
-      <c r="N53" t="n">
         <v>0.01014576812291071</v>
       </c>
     </row>
@@ -2791,10 +2632,10 @@
         <v>0.0003134956057468941</v>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F54" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
@@ -2812,12 +2653,9 @@
         <v>0.01118348023838589</v>
       </c>
       <c r="L54" t="n">
-        <v>2345.205909090909</v>
+        <v>0.07502028820213624</v>
       </c>
       <c r="M54" t="n">
-        <v>0.07502028820213624</v>
-      </c>
-      <c r="N54" t="n">
         <v>0.01145064578895998</v>
       </c>
     </row>
@@ -2835,10 +2673,10 @@
         <v>0.001696892368081793</v>
       </c>
       <c r="E55" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F55" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G55" t="n">
         <v>0</v>
@@ -2856,12 +2694,9 @@
         <v>0.01163548500161182</v>
       </c>
       <c r="L55" t="n">
-        <v>2571.986</v>
+        <v>0.06534536574321148</v>
       </c>
       <c r="M55" t="n">
-        <v>0.06534536574321148</v>
-      </c>
-      <c r="N55" t="n">
         <v>0.006556948109287463</v>
       </c>
     </row>
@@ -2879,10 +2714,10 @@
         <v>0.001307152701005343</v>
       </c>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F56" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -2900,12 +2735,9 @@
         <v>0.01106269242654978</v>
       </c>
       <c r="L56" t="n">
-        <v>2617.182380952381</v>
+        <v>0.05314065824197534</v>
       </c>
       <c r="M56" t="n">
-        <v>0.05314065824197534</v>
-      </c>
-      <c r="N56" t="n">
         <v>0.01108228186258304</v>
       </c>
     </row>
@@ -2923,10 +2755,10 @@
         <v>0.001785711492399367</v>
       </c>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="F57" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -2944,12 +2776,9 @@
         <v>0.01088235925124281</v>
       </c>
       <c r="L57" t="n">
-        <v>2762.37380952381</v>
+        <v>0.02779114754218814</v>
       </c>
       <c r="M57" t="n">
-        <v>0.02779114754218814</v>
-      </c>
-      <c r="N57" t="n">
         <v>0.007154773771056045</v>
       </c>
     </row>
@@ -2967,10 +2796,10 @@
         <v>0.00120259194874528</v>
       </c>
       <c r="E58" t="n">
+        <v>7.785714285714286</v>
+      </c>
+      <c r="F58" t="n">
         <v>0.4629100498862758</v>
-      </c>
-      <c r="F58" t="n">
-        <v>7.5</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -2988,12 +2817,9 @@
         <v>0.0108375906924234</v>
       </c>
       <c r="L58" t="n">
-        <v>2908.158095238095</v>
+        <v>0.1000633516229827</v>
       </c>
       <c r="M58" t="n">
-        <v>0.1000633516229827</v>
-      </c>
-      <c r="N58" t="n">
         <v>0.006923863932131116</v>
       </c>
     </row>
@@ -3011,10 +2837,10 @@
         <v>-0.00110218248522409</v>
       </c>
       <c r="E59" t="n">
+        <v>10.47826086956522</v>
+      </c>
+      <c r="F59" t="n">
         <v>1.774044306543957</v>
-      </c>
-      <c r="F59" t="n">
-        <v>7.785714285714286</v>
       </c>
       <c r="G59" t="n">
         <v>0.4629100498862758</v>
@@ -3032,12 +2858,9 @@
         <v>0.01057987722739018</v>
       </c>
       <c r="L59" t="n">
-        <v>3133.713043478261</v>
+        <v>0.04342780672605739</v>
       </c>
       <c r="M59" t="n">
-        <v>0.04342780672605739</v>
-      </c>
-      <c r="N59" t="n">
         <v>0.00951787448053463</v>
       </c>
     </row>
@@ -3055,10 +2878,10 @@
         <v>0.003352439413839559</v>
       </c>
       <c r="E60" t="n">
+        <v>12.47619047619048</v>
+      </c>
+      <c r="F60" t="n">
         <v>0.5117663157191586</v>
-      </c>
-      <c r="F60" t="n">
-        <v>10.47826086956522</v>
       </c>
       <c r="G60" t="n">
         <v>1.774044306543957</v>
@@ -3076,12 +2899,9 @@
         <v>0.01079650282484135</v>
       </c>
       <c r="L60" t="n">
-        <v>3133.929047619047</v>
+        <v>-0.03035573367168509</v>
       </c>
       <c r="M60" t="n">
-        <v>-0.03035573367168509</v>
-      </c>
-      <c r="N60" t="n">
         <v>0.009992448196891199</v>
       </c>
     </row>
@@ -3099,10 +2919,10 @@
         <v>-0.001663202274213349</v>
       </c>
       <c r="E61" t="n">
+        <v>13.18181818181818</v>
+      </c>
+      <c r="F61" t="n">
         <v>0.5884898863364998</v>
-      </c>
-      <c r="F61" t="n">
-        <v>12.47619047619048</v>
       </c>
       <c r="G61" t="n">
         <v>0.5117663157191586</v>
@@ -3120,12 +2940,9 @@
         <v>0.01087562686136523</v>
       </c>
       <c r="L61" t="n">
-        <v>3205.678181818182</v>
+        <v>0.02191339992912611</v>
       </c>
       <c r="M61" t="n">
-        <v>0.02191339992912611</v>
-      </c>
-      <c r="N61" t="n">
         <v>0.005553043853541538</v>
       </c>
     </row>
@@ -3143,10 +2960,10 @@
         <v>-0.0001793981139665002</v>
       </c>
       <c r="E62" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F62" t="n">
-        <v>13.18181818181818</v>
+        <v>0</v>
       </c>
       <c r="G62" t="n">
         <v>0.5884898863364998</v>
@@ -3164,12 +2981,9 @@
         <v>0.0118021176538321</v>
       </c>
       <c r="L62" t="n">
-        <v>3214.292727272727</v>
+        <v>-0.01270224417748833</v>
       </c>
       <c r="M62" t="n">
-        <v>-0.01270224417748833</v>
-      </c>
-      <c r="N62" t="n">
         <v>0.004823547712956068</v>
       </c>
     </row>
@@ -3187,10 +3001,10 @@
         <v>-0.001370933546374631</v>
       </c>
       <c r="E63" t="n">
+        <v>15.47619047619048</v>
+      </c>
+      <c r="F63" t="n">
         <v>0.5117663157191586</v>
-      </c>
-      <c r="F63" t="n">
-        <v>15</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -3208,12 +3022,9 @@
         <v>0.01319854398093612</v>
       </c>
       <c r="L63" t="n">
-        <v>3079.2</v>
+        <v>-0.01374157063797421</v>
       </c>
       <c r="M63" t="n">
-        <v>-0.01374157063797421</v>
-      </c>
-      <c r="N63" t="n">
         <v>0.007902074550866342</v>
       </c>
     </row>
@@ -3231,10 +3042,10 @@
         <v>0.003336168774512371</v>
       </c>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F64" t="n">
-        <v>15.47619047619048</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
         <v>0.5117663157191586</v>
@@ -3252,12 +3063,9 @@
         <v>0.01268992279066627</v>
       </c>
       <c r="L64" t="n">
-        <v>3169.565714285714</v>
+        <v>0.02682231018168002</v>
       </c>
       <c r="M64" t="n">
-        <v>0.02682231018168002</v>
-      </c>
-      <c r="N64" t="n">
         <v>0.00367085582850395</v>
       </c>
     </row>
@@ -3275,10 +3083,10 @@
         <v>0.00300836565616458</v>
       </c>
       <c r="E65" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F65" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G65" t="n">
         <v>0</v>
@@ -3296,12 +3104,9 @@
         <v>0.01185439844069469</v>
       </c>
       <c r="L65" t="n">
-        <v>3228.5705</v>
+        <v>0.008331553086947219</v>
       </c>
       <c r="M65" t="n">
-        <v>0.008331553086947219</v>
-      </c>
-      <c r="N65" t="n">
         <v>0.008436902185629019</v>
       </c>
     </row>
@@ -3319,10 +3124,10 @@
         <v>0.004852589564707133</v>
       </c>
       <c r="E66" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F66" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -3340,12 +3145,9 @@
         <v>0.01160480870949199</v>
       </c>
       <c r="L66" t="n">
-        <v>3298.3165</v>
+        <v>0.02016432686597325</v>
       </c>
       <c r="M66" t="n">
-        <v>0.02016432686597325</v>
-      </c>
-      <c r="N66" t="n">
         <v>0.004507068641549324</v>
       </c>
     </row>
@@ -3363,10 +3165,10 @@
         <v>0.007806462887876897</v>
       </c>
       <c r="E67" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F67" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
@@ -3384,12 +3186,9 @@
         <v>0.01127597440704098</v>
       </c>
       <c r="L67" t="n">
-        <v>3437.666956521739</v>
+        <v>0.03167731596145429</v>
       </c>
       <c r="M67" t="n">
-        <v>0.03167731596145429</v>
-      </c>
-      <c r="N67" t="n">
         <v>0.004640143868948452</v>
       </c>
     </row>
@@ -3407,10 +3206,10 @@
         <v>0.00682000560585494</v>
       </c>
       <c r="E68" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F68" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -3428,12 +3227,9 @@
         <v>0.01100183258734555</v>
       </c>
       <c r="L68" t="n">
-        <v>3410.02</v>
+        <v>-0.06553910590996359</v>
       </c>
       <c r="M68" t="n">
-        <v>-0.06553910590996359</v>
-      </c>
-      <c r="N68" t="n">
         <v>0.00911906705470609</v>
       </c>
     </row>
@@ -3451,10 +3247,10 @@
         <v>0.004450448384288208</v>
       </c>
       <c r="E69" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F69" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
@@ -3472,12 +3268,9 @@
         <v>0.01128989574866712</v>
       </c>
       <c r="L69" t="n">
-        <v>3154.45947368421</v>
+        <v>0.004119156305110394</v>
       </c>
       <c r="M69" t="n">
-        <v>0.004119156305110394</v>
-      </c>
-      <c r="N69" t="n">
         <v>0.01501736629962732</v>
       </c>
     </row>
@@ -3495,10 +3288,10 @@
         <v>0.006776740301411177</v>
       </c>
       <c r="E70" t="n">
+        <v>16.26086956521739</v>
+      </c>
+      <c r="F70" t="n">
         <v>0.6887004431501822</v>
-      </c>
-      <c r="F70" t="n">
-        <v>16</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -3516,12 +3309,9 @@
         <v>0.01115788972180143</v>
       </c>
       <c r="L70" t="n">
-        <v>3032.401304347826</v>
+        <v>-0.07642670399442597</v>
       </c>
       <c r="M70" t="n">
-        <v>-0.07642670399442597</v>
-      </c>
-      <c r="N70" t="n">
         <v>0.01345981402579843</v>
       </c>
     </row>
@@ -3539,10 +3329,10 @@
         <v>0.001721120601488879</v>
       </c>
       <c r="E71" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F71" t="n">
-        <v>16.26086956521739</v>
+        <v>0</v>
       </c>
       <c r="G71" t="n">
         <v>0.6887004431501822</v>
@@ -3560,12 +3350,9 @@
         <v>0.01168668720803856</v>
       </c>
       <c r="L71" t="n">
-        <v>2799.536818181818</v>
+        <v>-0.09720713018063898</v>
       </c>
       <c r="M71" t="n">
-        <v>-0.09720713018063898</v>
-      </c>
-      <c r="N71" t="n">
         <v>0.01423401624295071</v>
       </c>
     </row>
@@ -3583,10 +3370,10 @@
         <v>0.01113291156191121</v>
       </c>
       <c r="E72" t="n">
+        <v>18.52380952380953</v>
+      </c>
+      <c r="F72" t="n">
         <v>0.5117663157191595</v>
-      </c>
-      <c r="F72" t="n">
-        <v>18</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
@@ -3604,12 +3391,9 @@
         <v>0.01126595562931354</v>
       </c>
       <c r="L72" t="n">
-        <v>2720.719047619048</v>
+        <v>0.1227824774957074</v>
       </c>
       <c r="M72" t="n">
-        <v>0.1227824774957074</v>
-      </c>
-      <c r="N72" t="n">
         <v>0.01756016039991735</v>
       </c>
     </row>
@@ -3627,10 +3411,10 @@
         <v>0.008966594503365899</v>
       </c>
       <c r="E73" t="n">
+        <v>19.34782608695652</v>
+      </c>
+      <c r="F73" t="n">
         <v>0.7751067757631785</v>
-      </c>
-      <c r="F73" t="n">
-        <v>18.52380952380953</v>
       </c>
       <c r="G73" t="n">
         <v>0.5117663157191595</v>
@@ -3648,12 +3432,9 @@
         <v>0.01192325535589123</v>
       </c>
       <c r="L73" t="n">
-        <v>2733.913913043478</v>
+        <v>-0.09025332333637748</v>
       </c>
       <c r="M73" t="n">
-        <v>-0.09025332333637748</v>
-      </c>
-      <c r="N73" t="n">
         <v>0.01141310886295815</v>
       </c>
     </row>
@@ -3671,10 +3452,10 @@
         <v>0.007316411660442057</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F74" t="n">
-        <v>19.34782608695652</v>
+        <v>0</v>
       </c>
       <c r="G74" t="n">
         <v>0.7751067757631785</v>
@@ -3692,12 +3473,9 @@
         <v>0.01193152057448166</v>
       </c>
       <c r="L74" t="n">
-        <v>2634.62</v>
+        <v>0.001277813812041062</v>
       </c>
       <c r="M74" t="n">
-        <v>0.001277813812041062</v>
-      </c>
-      <c r="N74" t="n">
         <v>0.0164496972700753</v>
       </c>
     </row>
@@ -3715,10 +3493,10 @@
         <v>0.001577287422393159</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F75" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -3736,12 +3514,9 @@
         <v>0.01233830370713318</v>
       </c>
       <c r="L75" t="n">
-        <v>2583.033636363636</v>
+        <v>0.1145457216419123</v>
       </c>
       <c r="M75" t="n">
-        <v>0.1145457216419123</v>
-      </c>
-      <c r="N75" t="n">
         <v>0.02487247818140731</v>
       </c>
     </row>
@@ -3759,10 +3534,10 @@
         <v>0.003209288265454191</v>
       </c>
       <c r="E76" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F76" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -3780,12 +3555,9 @@
         <v>0.01276910238125395</v>
       </c>
       <c r="L76" t="n">
-        <v>2895.459</v>
+        <v>0.04228389605798122</v>
       </c>
       <c r="M76" t="n">
-        <v>0.04228389605798122</v>
-      </c>
-      <c r="N76" t="n">
         <v>0.01354688819517796</v>
       </c>
     </row>
@@ -3803,10 +3575,10 @@
         <v>0.003908377089340664</v>
       </c>
       <c r="E77" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F77" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
@@ -3824,12 +3596,9 @@
         <v>0.01281207157693998</v>
       </c>
       <c r="L77" t="n">
-        <v>3145.586</v>
+        <v>0.09374369910155589</v>
       </c>
       <c r="M77" t="n">
-        <v>0.09374369910155589</v>
-      </c>
-      <c r="N77" t="n">
         <v>0.0180203901375043</v>
       </c>
     </row>
@@ -3847,10 +3616,10 @@
         <v>0.008160115097238574</v>
       </c>
       <c r="E78" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F78" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
         <v>0</v>
@@ -3868,12 +3637,9 @@
         <v>0.01281902591865447</v>
       </c>
       <c r="L78" t="n">
-        <v>3175.607142857143</v>
+        <v>-0.04207926300095677</v>
       </c>
       <c r="M78" t="n">
-        <v>-0.04207926300095677</v>
-      </c>
-      <c r="N78" t="n">
         <v>0.01398660657956558</v>
       </c>
     </row>
@@ -3891,10 +3657,10 @@
         <v>0.009088214708421694</v>
       </c>
       <c r="E79" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F79" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
         <v>0</v>
@@ -3912,12 +3678,9 @@
         <v>0.01234012412924823</v>
       </c>
       <c r="L79" t="n">
-        <v>2870.904545454545</v>
+        <v>-0.01550382366930569</v>
       </c>
       <c r="M79" t="n">
-        <v>-0.01550382366930569</v>
-      </c>
-      <c r="N79" t="n">
         <v>0.01936594170509362</v>
       </c>
     </row>
@@ -3935,10 +3698,10 @@
         <v>0.01127143524965879</v>
       </c>
       <c r="E80" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F80" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -3956,12 +3719,9 @@
         <v>0.01210951789996662</v>
       </c>
       <c r="L80" t="n">
-        <v>2824.417</v>
+        <v>-0.00277435047766772</v>
       </c>
       <c r="M80" t="n">
-        <v>-0.00277435047766772</v>
-      </c>
-      <c r="N80" t="n">
         <v>0.01854433821511479</v>
       </c>
     </row>
@@ -3979,10 +3739,10 @@
         <v>0.01082884470775469</v>
       </c>
       <c r="E81" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="F81" t="n">
         <v>0.4442616583193181</v>
-      </c>
-      <c r="F81" t="n">
-        <v>21</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -4000,12 +3760,9 @@
         <v>0.01219430351518236</v>
       </c>
       <c r="L81" t="n">
-        <v>2784.32</v>
+        <v>0.006258680340817113</v>
       </c>
       <c r="M81" t="n">
-        <v>0.006258680340817113</v>
-      </c>
-      <c r="N81" t="n">
         <v>0.01054418667519808</v>
       </c>
     </row>
@@ -4023,10 +3780,10 @@
         <v>0.0124843064618787</v>
       </c>
       <c r="E82" t="n">
+        <v>19.65217391304348</v>
+      </c>
+      <c r="F82" t="n">
         <v>0.7751067757631785</v>
-      </c>
-      <c r="F82" t="n">
-        <v>20.25</v>
       </c>
       <c r="G82" t="n">
         <v>0.4442616583193181</v>
@@ -4044,12 +3801,9 @@
         <v>0.01171880240956247</v>
       </c>
       <c r="L82" t="n">
-        <v>2768.78</v>
+        <v>-0.04083638763674158</v>
       </c>
       <c r="M82" t="n">
-        <v>-0.04083638763674158</v>
-      </c>
-      <c r="N82" t="n">
         <v>0.01390505859545336</v>
       </c>
     </row>
@@ -4067,10 +3821,10 @@
         <v>0.007806784982991033</v>
       </c>
       <c r="E83" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F83" t="n">
-        <v>19.65217391304348</v>
+        <v>0</v>
       </c>
       <c r="G83" t="n">
         <v>0.7751067757631785</v>
@@ -4088,12 +3842,9 @@
         <v>0.0125065769025734</v>
       </c>
       <c r="L83" t="n">
-        <v>2899.633809523809</v>
+        <v>0.062830372656691</v>
       </c>
       <c r="M83" t="n">
-        <v>0.062830372656691</v>
-      </c>
-      <c r="N83" t="n">
         <v>0.01315300536851439</v>
       </c>
     </row>
@@ -4111,10 +3862,10 @@
         <v>0.01636501665230972</v>
       </c>
       <c r="E84" t="n">
+        <v>17.45454545454545</v>
+      </c>
+      <c r="F84" t="n">
         <v>0.509647191437626</v>
-      </c>
-      <c r="F84" t="n">
-        <v>18</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -4132,12 +3883,9 @@
         <v>0.01149633221713131</v>
       </c>
       <c r="L84" t="n">
-        <v>2813.168181818182</v>
+        <v>-0.07009771490524663</v>
       </c>
       <c r="M84" t="n">
-        <v>-0.07009771490524663</v>
-      </c>
-      <c r="N84" t="n">
         <v>0.009192618189897639</v>
       </c>
     </row>
@@ -4155,10 +3903,10 @@
         <v>0.008315963041594987</v>
       </c>
       <c r="E85" t="n">
+        <v>16.89130434782609</v>
+      </c>
+      <c r="F85" t="n">
         <v>0.2108705839183244</v>
-      </c>
-      <c r="F85" t="n">
-        <v>17.45454545454545</v>
       </c>
       <c r="G85" t="n">
         <v>0.509647191437626</v>
@@ -4176,12 +3924,9 @@
         <v>0.01104341958050647</v>
       </c>
       <c r="L85" t="n">
-        <v>2595.877391304348</v>
+        <v>-0.04610444801208813</v>
       </c>
       <c r="M85" t="n">
-        <v>-0.04610444801208813</v>
-      </c>
-      <c r="N85" t="n">
         <v>0.02149344746084847</v>
       </c>
     </row>
@@ -4199,10 +3944,10 @@
         <v>0.00670339113745233</v>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
+        <v>16.5</v>
       </c>
       <c r="F86" t="n">
-        <v>16.89130434782609</v>
+        <v>0</v>
       </c>
       <c r="G86" t="n">
         <v>0.2108705839183244</v>
@@ -4220,12 +3965,9 @@
         <v>0.01134099625171792</v>
       </c>
       <c r="L86" t="n">
-        <v>2591.471</v>
+        <v>0.05676245528416768</v>
       </c>
       <c r="M86" t="n">
-        <v>0.05676245528416768</v>
-      </c>
-      <c r="N86" t="n">
         <v>0.0136388534842457</v>
       </c>
     </row>
@@ -4243,10 +3985,10 @@
         <v>0.007395837090733215</v>
       </c>
       <c r="E87" t="n">
+        <v>16.34090909090909</v>
+      </c>
+      <c r="F87" t="n">
         <v>0.2383656473113982</v>
-      </c>
-      <c r="F87" t="n">
-        <v>16.5</v>
       </c>
       <c r="G87" t="n">
         <v>0</v>
@@ -4264,12 +4006,9 @@
         <v>0.01137529276183336</v>
       </c>
       <c r="L87" t="n">
-        <v>2723.151363636364</v>
+        <v>0.02965838335944748</v>
       </c>
       <c r="M87" t="n">
-        <v>0.02965838335944748</v>
-      </c>
-      <c r="N87" t="n">
         <v>0.007652214389754769</v>
       </c>
     </row>
@@ -4287,10 +4026,10 @@
         <v>0.008400019543973736</v>
       </c>
       <c r="E88" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F88" t="n">
-        <v>16.34090909090909</v>
+        <v>0</v>
       </c>
       <c r="G88" t="n">
         <v>0.2383656473113982</v>
@@ -4302,12 +4041,9 @@
         <v>0.01134762103812315</v>
       </c>
       <c r="L88" t="n">
-        <v>2747.612631578947</v>
+        <v>0.009303287161463558</v>
       </c>
       <c r="M88" t="n">
-        <v>0.009303287161463558</v>
-      </c>
-      <c r="N88" t="n">
         <v>0.005962446576861836</v>
       </c>
     </row>
@@ -4323,10 +4059,10 @@
         <v>-0.004502363615381477</v>
       </c>
       <c r="E89" t="n">
+        <v>15.83333333333333</v>
+      </c>
+      <c r="F89" t="n">
         <v>0.2439750182371336</v>
-      </c>
-      <c r="F89" t="n">
-        <v>16</v>
       </c>
       <c r="G89" t="n">
         <v>0</v>
@@ -4336,12 +4072,9 @@
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="n">
-        <v>2761.764</v>
+        <v>0.004348831161325784</v>
       </c>
       <c r="M89" t="n">
-        <v>0.004348831161325784</v>
-      </c>
-      <c r="N89" t="n">
         <v>0.006707859815548966</v>
       </c>
     </row>

</xml_diff>